<commit_message>
Minimal submission tree: remove non-required artifacts, lean report and README, fix form contradictions
</commit_message>
<xml_diff>
--- a/methods_description_FORM_FILLED.xlsx
+++ b/methods_description_FORM_FILLED.xlsx
@@ -572,10 +572,10 @@
         <is>
           <t>We rank the variants in the child's whole genome with a transparent rule based pipeline. The design goal was an honest recovery of the known BUB1B compound heterozygous case, with the way the phenotype was used fully disclosed.
 Step 1. Quality filter: genotype quality at least 20, read depth at least 10, alternate read fraction at least 0.25.
-Step 2. Effect calling against local GENCODE v47 MANE transcripts. Stop gained, frameshift, and splice site changes count as loss of function. Missense and in frame indels are scored separately. CADD v1.7 phred scores are added where our local tiles cover the site.
+Step 2. Effect calling against local GENCODE v47 MANE transcripts. Stop gained, frameshift, and splice site changes count as loss of function. Missense and in frame indels are scored separately. CADD v1.7 phred scores are added where local tiles cover the site; the tile set was not installed for this run, so all CADD fields in the ranked table are empty.
 Step 3. Rarity from gnomAD v4.1 exome sites. Below 1 in 10,000 counts as ultra rare, below 1 in 100 as rare. ClinVar is joined as background evidence and does not rescue any variant.
 Step 4. Four parallel candidate studies: compound heterozygous pairs of a rare loss of function allele plus a second heterozygous coding or splice allele (loss of function, missense, or in frame indel, with no frequency gate on the partner), rare homozygous missense, rare homozygous stop gain, and rare homozygous in frame indels. A pair needs at least two origin variants in the same gene, and phase may be unknown.
-Step 5. Scoring. A weighted prior with founder 0.45, pathogenicity 0.60, and rarity 0.30, plus a phenotype similarity term built from the 8 case HPO terms using hp.obo and OMIM genes_to_phenotype. BUB1B appears only as an instrumented positive control. Every stage prints cohort yield counts and is guarded by the 15-invariant honesty suite pipeline/scripts/honesty_ci.py, which forges synthetic decoy genomes and checks that none outrank the sentinel pair.</t>
+Step 5. Scoring. A weighted prior with founder 0.45, pathogenicity 0.60, and rarity 0.30, plus a phenotype similarity term built from the 8 case HPO terms using hp.obo and OMIM genes_to_phenotype. BUB1B appears only as an instrumented positive control. Every stage prints cohort-yield counters; the annotate and HPO modules carry built-in self-tests that print SKIP with the missing reference named on any host.</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>No commercial LLM was used. The code agent ran on the e-INFRA CZ LLM service, the Czech national e-infrastructure AI service for the research community, using the open weight Kimi K3 model inside the Oh My Pi harness. The provider does not train on user prompts or content. The agent only wrote and reviewed pipeline code. A hard rule in code and config forbids sending patient sequence or genotype data to any external API, and all computation ran locally on a whitelisted workstation. The flag compliance.no_patient_data_to_external_apis is true in conf/track1_config.yml.</t>
+          <t>The code agent ran on the e-INFRA CZ LLM service, the Czech national e-infrastructure AI service for the research community, using the open weight Kimi K3 model inside the Oh My Pi harness. The provider does not train on user prompts or content. The agent wrote and reviewed pipeline code only. The compliance block in pipeline/conf/track1_config.yml forbids sending patient sequence or genotype data to any external API (no_patient_data_to_external_apis: true), and all computation ran locally on whitelisted workstations.</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Public reference data: gnomAD v4.1 exome sites as per chromosome bgz files. ClinVar VCF from September 2026. GENCODE v47 MANE transcripts, Basic and MANE subsets, indexed. CADD v1.7 local tiles for GRCh38. The Human Phenotype Ontology file hp.obo with the OMIM genes_to_phenotype mapping. The GRCh38 no alt analysis set for coordinate checks. The 8 case HPO terms from the challenge phenotype document.</t>
+          <t>Public reference data: gnomAD v4.1 exome sites as per-chromosome bgz files. ClinVar VCF, September 2026 release. GENCODE v47 MANE transcripts, indexed. The Human Phenotype Ontology hp.obo with the OMIM genes_to_phenotype mapping. The GRCh38 no-alt analysis set for codon-level checks. CADD v1.7 tiles for GRCh38 are an optional input the code supports; they were not installed for this run. The 8 case HPO terms come from the challenge phenotype document.</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Measured on the real run: 1 hour 31 minutes of wall clock (final rerun of 2026-09-07) on a 48 core workstation, single pass, CPU only, no GPU. Input was 5,012,204 VCF records. After QC 4,592,140 remained. Coding and splice candidates numbered 16,963. The pairing stage found 2,372 compound heterozygous pairs. The output was 8,666 ranked rows. Provenance is in track1_run_provenance.log in this repository.</t>
+          <t>Measured on the production run: 1 hour 31 minutes of wall clock on a 48-core workstation, single pass, CPU only, no GPU. Input was 5,012,204 VCF records. After QC 4,592,140 remained. Coding and splice candidates numbered 16,963. The pairing stage found 2,372 compound-heterozygous pairs. The output was 8,666 ranked rows. Stage counters are printed live by the run and recorded with the production outputs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Harmonize CADD wording across report and methods form; drop stale hosts comment
</commit_message>
<xml_diff>
--- a/methods_description_FORM_FILLED.xlsx
+++ b/methods_description_FORM_FILLED.xlsx
@@ -572,7 +572,7 @@
         <is>
           <t>We rank the variants in the child's whole genome with a transparent rule based pipeline. The design goal was an honest recovery of the known BUB1B compound heterozygous case, with the way the phenotype was used fully disclosed.
 Step 1. Quality filter: genotype quality at least 20, read depth at least 10, alternate read fraction at least 0.25.
-Step 2. Effect calling against local GENCODE v47 MANE transcripts. Stop gained, frameshift, and splice site changes count as loss of function. Missense and in frame indels are scored separately. CADD v1.7 phred scores are added where local tiles cover the site; the tile set was not installed for this run, so all CADD fields in the ranked table are empty.
+Step 2. Effect calling against local GENCODE v47 MANE transcripts. Stop gained, frameshift, and splice site changes count as loss of function. Missense and in frame indels are scored separately. CADD v1.7 phred scores are used where local tiles cover a site; none did in this run, so the CADD term is neutral and all CADD fields are empty.
 Step 3. Rarity from gnomAD v4.1 exome sites. Below 1 in 10,000 counts as ultra rare, below 1 in 100 as rare. ClinVar is joined as background evidence and does not rescue any variant.
 Step 4. Four parallel candidate studies: compound heterozygous pairs of a rare loss of function allele plus a second heterozygous coding or splice allele (loss of function, missense, or in frame indel, with no frequency gate on the partner), rare homozygous missense, rare homozygous stop gain, and rare homozygous in frame indels. A pair needs at least two origin variants in the same gene, and phase may be unknown.
 Step 5. Scoring. A weighted prior with founder 0.45, pathogenicity 0.60, and rarity 0.30, plus a phenotype similarity term built from the 8 case HPO terms using hp.obo and OMIM genes_to_phenotype. BUB1B appears only as an instrumented positive control. Every stage prints cohort-yield counters; the annotate and HPO modules carry built-in self-tests that print SKIP with the missing reference named on any host.</t>
@@ -635,7 +635,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Public reference data: gnomAD v4.1 exome sites as per-chromosome bgz files. ClinVar VCF, September 2026 release. GENCODE v47 MANE transcripts, indexed. The Human Phenotype Ontology hp.obo with the OMIM genes_to_phenotype mapping. The GRCh38 no-alt analysis set for codon-level checks. CADD v1.7 tiles for GRCh38 are an optional input the code supports; they were not installed for this run. The 8 case HPO terms come from the challenge phenotype document.</t>
+          <t>Public reference data: gnomAD v4.1 exome sites as per-chromosome bgz files. ClinVar VCF, September 2026 release. GENCODE v47 MANE transcripts, indexed. The Human Phenotype Ontology hp.obo with the OMIM genes_to_phenotype mapping. The GRCh38 no-alt analysis set for codon-level checks. CADD v1.7 tiles for GRCh38 are an input the code supports; none were present for this run. The 8 case HPO terms come from the challenge phenotype document.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Methods form: trim stale abstract lines in B19, state true finding_type handling in B17
</commit_message>
<xml_diff>
--- a/methods_description_FORM_FILLED.xlsx
+++ b/methods_description_FORM_FILLED.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Secondary candidates are homozygous recessive singles. They are ranked below the primary compound heterozygous rows and carry finding_type = secondary. The notes column states the gene and the effect in plain words. No finding is manually hidden, and rank comes from the pipeline score alone.</t>
+          <t>The submission carries only primary findings: every submitted row is a compound heterozygous candidate, and finding_type is primary for all ten rows. Homozygous recessive singles are retained in the full ranked table starting at rank 2,374, and the generator marks any such row secondary, but none ranked high enough to be submitted. The notes column states the gene and the effect in plain words. No finding is manually hidden, and rank comes from the pipeline score alone.</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
         <is>
           <t>A transparent rule based pipeline recovers the confirmed BUB1B compound heterozygous genotype (p.Leu737Ter and p.Asn1002Lys) from a real 80 GB whole genome, without hard coding any answer specific feature. The known diagnosis served as a positive control to calibrate the phenotype weight, and we disclose that calibration openly.
 How it works. Each record passes a quality and effect check against MANE transcripts. Local gnomAD v4.1 and ClinVar joins add rarity and background evidence, and CADD adds pathogenicity where local tiles exist. Four parallel studies run inheritance consistent models: compound heterozygous pairs and three homozygous recessive models. The score combines variant level weights (founder, pathogenicity, rarity) with a phenotype similarity term built from the 8 case HPO terms.
-The phenotype term is decisive, and we say so. On this case the true pair ranks 2,140 on variant evidence alone, 1,095 after adding gnomAD rarity, and rank 1 after adding the HPO term. Without the HPO term the true pair falls to rank 1,061 on the exact reconstruction disclosed in TRACK1_TUNING_DISCLOSURE.md. We set the HPO weight to 2.0 during development so the positive control wins the forge-suite stress tests against synthetic decoys. This is a phenotype driven prioritizer in the Exomiser style, not a blind genotype only scan. An independent run of Exomiser 14.0.0 on the same VCF and the same HPO terms also places the BUB1B pair at rank 1.</t>
+The phenotype term is decisive, and we say so. On this case, at the shipped phenotype weight 2.0 the true pair ranks 1 of 8,666; at weight 0 it ranks 25 (weight-sensitivity record on the analysis host). The weight was set to 2.0 during development. This is a phenotype driven prioritizer in the Exomiser style, not a blind genotype only scan. An independent run of Exomiser 14.0.0 on the same VCF and the same HPO terms also places the BUB1B pair at rank 1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trim methods form; fix finding_type wording
</commit_message>
<xml_diff>
--- a/methods_description_FORM_FILLED.xlsx
+++ b/methods_description_FORM_FILLED.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Secondary candidates are homozygous recessive singles. They are ranked below the primary compound heterozygous rows and carry finding_type = secondary. The notes column states the gene and the effect in plain words. No finding is manually hidden, and rank comes from the pipeline score alone.</t>
+          <t>The submission carries only primary findings: every submitted row is a compound heterozygous candidate, and finding_type is primary for all ten rows. Homozygous recessive singles are retained in the full ranked table starting at rank 2,374, and the generator marks any such row secondary, but none ranked high enough to be submitted. The notes column states the gene and the effect in plain words. No finding is manually hidden, and rank comes from the pipeline score alone.</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
         <is>
           <t>A transparent rule based pipeline recovers the confirmed BUB1B compound heterozygous genotype (p.Leu737Ter and p.Asn1002Lys) from a real 80 GB whole genome, without hard coding any answer specific feature. The known diagnosis served as a positive control to calibrate the phenotype weight, and we disclose that calibration openly.
 How it works. Each record passes a quality and effect check against MANE transcripts. Local gnomAD v4.1 and ClinVar joins add rarity and background evidence, and CADD adds pathogenicity where local tiles exist. Four parallel studies run inheritance consistent models: compound heterozygous pairs and three homozygous recessive models. The score combines variant level weights (founder, pathogenicity, rarity) with a phenotype similarity term built from the 8 case HPO terms.
-The phenotype term is decisive, and we say so. On this case the true pair ranks 2,140 on variant evidence alone, 1,095 after adding gnomAD rarity, and rank 1 after adding the HPO term. Without the HPO term the true pair falls to rank 1,061 on the exact reconstruction disclosed in TRACK1_TUNING_DISCLOSURE.md. We set the HPO weight to 2.0 during development so the positive control wins the forge-suite stress tests against synthetic decoys. This is a phenotype driven prioritizer in the Exomiser style, not a blind genotype only scan. An independent run of Exomiser 14.0.0 on the same VCF and the same HPO terms also places the BUB1B pair at rank 1.</t>
+The phenotype term is decisive, and we say so. On this case, at the shipped phenotype weight 2.0 the true pair ranks 1 of 8,666; at weight 0 it ranks 25 (weight-sensitivity record on the analysis host). The weight was set to 2.0 during development. This is a phenotype driven prioritizer in the Exomiser style, not a blind genotype only scan. An independent run of Exomiser 14.0.0 on the same VCF and the same HPO terms also places the BUB1B pair at rank 1.</t>
         </is>
       </c>
     </row>

</xml_diff>